<commit_message>
Make "did you fix all of them?" a machine question
The founder asked whether the new standard reached every row or just the one
he opened. The honest answer was yes - but I had to go and check, and a
standard nobody checks is a standard that gets applied to whatever row
someone happened to be looking at.

The builder now prints a coverage line on every regeneration, and tests each
documented row against the four rules the standard is made of: possible
answers listed, formula written as real rules, source naming a file/feed/
field rather than "the account record", variables written raw to ours.

  COVERAGE: 53 of 158 rows documented, 105 not yet written
  every documented row meets the standard

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Calculation Module/calculation-inventory-v1.xlsx
+++ b/Calculation Module/calculation-inventory-v1.xlsx
@@ -118,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -149,9 +149,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -724,7 +721,7 @@
     <row r="1" ht="46" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CALCULATION INVENTORY · Phase 1 — Net worth, Performance and the 8 screens they open · 158 calculations · generated from commit 247201d on 2026-08-17  ⚠ TREE WAS DIRTY. EVERY FORMULA HERE DESCRIBES THE CODE AS IT IS TODAY, BUGS INCLUDED — you cannot fix what you have not described, and a probe can only execute what exists. Where the current behaviour is wrong, Status says DEFECT and the corrected version sits in WHAT IT SHOULD BE; the difference between those two columns is the work list. GREY columns are generated from the code and overwritten on every regeneration — never edit them. CREAM columns are written by hand and preserved. A row is not documented until its probe passes.</t>
+          <t>CALCULATION INVENTORY · Phase 1 — Net worth, Performance and the 8 screens they open · 158 calculations · generated from commit 09c3aaa on 2026-08-17  ⚠ TREE WAS DIRTY. EVERY FORMULA HERE DESCRIBES THE CODE AS IT IS TODAY, BUGS INCLUDED — you cannot fix what you have not described, and a probe can only execute what exists. Where the current behaviour is wrong, Status says DEFECT and the corrected version sits in WHAT IT SHOULD BE; the difference between those two columns is the work list. GREY columns are generated from the code and overwritten on every regeneration — never edit them. CREAM columns are written by hand and preserved. A row is not documented until its probe passes.</t>
         </is>
       </c>
     </row>
@@ -11781,7 +11778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -11819,57 +11816,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="12" t="inlineStr">
-        <is>
-          <t>The account id is first in the dedupe key. If a broker's internal account id changes between connections, every key changes and the whole history re-imports. Did the Vanguard account get disconnected and reconnected at any point?</t>
-        </is>
-      </c>
-      <c r="C3" s="12" t="inlineStr">
-        <is>
-          <t>This is the last standing explanation for the $1.4m of contributions Vanguard says never happened. Everything else has been ruled out by running the code: the activity mapping is correct, option trades stay internal, the dedupe set persists across syncs, and nothing in the connect flow writes opening rows.</t>
-        </is>
-      </c>
-      <c r="D3" s="12" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>You named FIVE asset classes. The code has SEVEN. Which do you want?
-Yours: Stocks and Funds · Bonds and CDs · Alternatives · Cash or Cash Equivalent · Personal Property.
-The code's: Cash · Bonds &amp; CDs · Stocks / ETFs · Alternatives · Real estate · Personal property · Unclassified.
-Two real differences: the code separates Real estate from Personal property (you have one class for both), and it has "Unclassified" for an account whose contents we were never told.</t>
-        </is>
-      </c>
-      <c r="C4" s="12" t="inlineStr">
-        <is>
-          <t>This is the top of the taxonomy — every total, every donut slice and every projection sits under it. It has to be settled before names are fixed, not after.</t>
-        </is>
-      </c>
-      <c r="D4" s="12" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>Your wording was "Cash or Cash Equivalent". A money-market fund IS a cash equivalent in ordinary usage — but your own rule of 2026-08-04 moved money-market funds OUT of cash and into Stocks / ETFs, so their dividends get measured. Is that rule still what you want?</t>
-        </is>
-      </c>
-      <c r="C5" s="12" t="inlineStr">
-        <is>
-          <t>It decides where VMFXX lands, which is the founder finding F6. The rules currently disagree with themselves: the class rule says measured, the on-screen grouping still says Cash.</t>
-        </is>
-      </c>
-      <c r="D5" s="12" t="inlineStr"/>
-    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>

</xml_diff>

<commit_message>
Claude's v2 caught a tax bug, and it is worse than he said
He challenged our long-term/short-term rule: the threshold is MORE THAN one
year counting from the day after purchase, so a sale on the anniversary is
short term where our ">= 12 whole months" calls it long. He described it as
being a day out.

Ran it. Our code never looks at the day at all - it subtracts calendar month
numbers. Buy on 31 January, sell on 1 January: 335 days held, reported as
LONG term. The error reaches a full month, and it always runs the same way,
toward the lower rate, which understates the tax bill - the mistake this
sheet itself calls the worse one.

capGains moves from PINNED to DEFECT with the day-count fix, plus two rules
worth adding while it is open: an inherited holding is long-term however
briefly held, which matters at this audience's age, and a wash sale extends
the holding period.

2043 green.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Calculation Module/calculation-inventory-v1.xlsx
+++ b/Calculation Module/calculation-inventory-v1.xlsx
@@ -5345,21 +5345,29 @@
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>probes/performance-lot-math.probe.test.ts</t>
+          <t>probes/holding-period.probe.test.ts</t>
         </is>
       </c>
       <c r="I62" s="24" t="inlineStr">
         <is>
-          <t>YOUR CALL</t>
-        </is>
-      </c>
-      <c r="J62" s="3" t="inlineStr"/>
+          <t>DEFECT</t>
+        </is>
+      </c>
+      <c r="J62" s="3" t="inlineStr">
+        <is>
+          <t>A gain is long-term only when the shares were held MORE THAN one year, counting from the day AFTER purchase. Sold on the one-year anniversary is SHORT term.</t>
+        </is>
+      </c>
       <c r="K62" s="3" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L62" s="3" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L62" s="3" t="inlineStr">
+        <is>
+          <t>Found by Claude's v2 review, and it is worse than he described. Our code never looks at the DAY — it subtracts calendar month numbers, so anything bought in January and sold the following January counts as a full year however late in the month it was bought. Buy on 31 January, sell on 1 January: 335 days held, reported LONG term. The error reaches a full month and always runs the same way — toward the lower tax rate, which understates the bill, the mistake this sheet itself calls the worse one. FIX: count actual days. Long-term is more than 365 days from the day after purchase. Roughly ten minutes. Two further rules worth adding while it is open: an inherited holding is long-term however briefly it was held (common at this age), and a wash sale extends the holding period.</t>
+        </is>
+      </c>
       <c r="M62" s="5" t="inlineStr"/>
       <c r="N62" s="5" t="inlineStr"/>
       <c r="O62" s="6" t="inlineStr">

</xml_diff>